<commit_message>
fix: Correct the IranWar implementation
</commit_message>
<xml_diff>
--- a/factor_master.xlsx
+++ b/factor_master.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29911"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\bkrai\Source\risk\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{70C24323-A31A-4C54-B93E-7CDA9B3C5D23}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6EEB79B3-8A1F-4750-9F6C-F78A727D4C86}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" activeTab="10" xr2:uid="{C31FDC5B-A809-4BFD-99CB-DA02246721F7}"/>
   </bookViews>
@@ -92,7 +92,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2554" uniqueCount="724">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2549" uniqueCount="724">
   <si>
     <t>SPX</t>
   </si>
@@ -2360,111 +2360,7 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="47">
-    <dxf>
-      <border>
-        <top style="thin">
-          <color theme="0" tint="-0.24994659260841701"/>
-        </top>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <top style="thin">
-          <color theme="0" tint="-0.24994659260841701"/>
-        </top>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <top style="thin">
-          <color theme="0" tint="-0.24994659260841701"/>
-        </top>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <top style="thin">
-          <color theme="0" tint="-0.24994659260841701"/>
-        </top>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <bottom style="thin">
-          <color theme="0" tint="-0.24994659260841701"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color theme="0" tint="-0.24994659260841701"/>
-        </left>
-        <right style="thin">
-          <color theme="0" tint="-0.24994659260841701"/>
-        </right>
-        <top style="thin">
-          <color theme="0" tint="-0.24994659260841701"/>
-        </top>
-        <bottom style="thin">
-          <color theme="0" tint="-0.24994659260841701"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <top style="thin">
-          <color theme="0" tint="-0.24994659260841701"/>
-        </top>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <top style="thin">
-          <color theme="0" tint="-0.24994659260841701"/>
-        </top>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <top style="thin">
-          <color theme="0" tint="-0.24994659260841701"/>
-        </top>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <top style="thin">
-          <color theme="0" tint="-0.24994659260841701"/>
-        </top>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <top style="thin">
-          <color theme="0" tint="-0.24994659260841701"/>
-        </top>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
+  <dxfs count="39">
     <dxf>
       <border>
         <top style="thin">
@@ -2631,12 +2527,44 @@
       </font>
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
+    <dxf>
+      <border>
+        <top style="thin">
+          <color theme="0" tint="-0.24994659260841701"/>
+        </top>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <bottom style="thin">
+          <color theme="0" tint="-0.24994659260841701"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color theme="0" tint="-0.24994659260841701"/>
+        </left>
+        <right style="thin">
+          <color theme="0" tint="-0.24994659260841701"/>
+        </right>
+        <top style="thin">
+          <color theme="0" tint="-0.24994659260841701"/>
+        </top>
+        <bottom style="thin">
+          <color theme="0" tint="-0.24994659260841701"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
   </dxfs>
   <tableStyles count="1" defaultTableStyle="Table Style 1" defaultPivotStyle="PivotStyleLight16">
     <tableStyle name="Table Style 1" pivot="0" count="3" xr9:uid="{26B58CFA-74FB-41FD-AB02-EC6D3EA4F4A1}">
-      <tableStyleElement type="wholeTable" dxfId="5"/>
-      <tableStyleElement type="headerRow" dxfId="4"/>
-      <tableStyleElement type="firstRowStripe" size="3" dxfId="3"/>
+      <tableStyleElement type="wholeTable" dxfId="38"/>
+      <tableStyleElement type="headerRow" dxfId="37"/>
+      <tableStyleElement type="firstRowStripe" size="3" dxfId="36"/>
     </tableStyle>
   </tableStyles>
   <extLst>
@@ -2735,58 +2663,58 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{6DAD1482-C63D-400D-9F51-F22A8E35CAD8}" name="data" displayName="data" ref="A1:T107" totalsRowShown="0" headerRowDxfId="46" dataDxfId="45">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{6DAD1482-C63D-400D-9F51-F22A8E35CAD8}" name="data" displayName="data" ref="A1:T106" totalsRowShown="0" headerRowDxfId="35" dataDxfId="34">
   <tableColumns count="20">
-    <tableColumn id="1" xr3:uid="{740DC173-AAC9-4239-A44E-C43F8517304D}" name="asset_class" dataDxfId="44"/>
-    <tableColumn id="2" xr3:uid="{A3BC3BB8-0420-458E-AECD-FD567519FA40}" name="region" dataDxfId="43"/>
-    <tableColumn id="3" xr3:uid="{0E50B2E3-0362-41DB-ACC2-478CC6F618A4}" name="factor_name" dataDxfId="42"/>
-    <tableColumn id="11" xr3:uid="{C400A641-F032-4829-A2CD-62831D657B37}" name="source" dataDxfId="41"/>
-    <tableColumn id="12" xr3:uid="{BC682952-ADA8-4869-A16F-B9E7BC86E430}" name="diffusion_type" dataDxfId="40"/>
-    <tableColumn id="16" xr3:uid="{A99CC35E-FB67-451C-BF9C-DA8D933B1B0C}" name="multiplier" dataDxfId="39">
+    <tableColumn id="1" xr3:uid="{740DC173-AAC9-4239-A44E-C43F8517304D}" name="asset_class" dataDxfId="33"/>
+    <tableColumn id="2" xr3:uid="{A3BC3BB8-0420-458E-AECD-FD567519FA40}" name="region" dataDxfId="32"/>
+    <tableColumn id="3" xr3:uid="{0E50B2E3-0362-41DB-ACC2-478CC6F618A4}" name="factor_name" dataDxfId="31"/>
+    <tableColumn id="11" xr3:uid="{C400A641-F032-4829-A2CD-62831D657B37}" name="source" dataDxfId="30"/>
+    <tableColumn id="12" xr3:uid="{BC682952-ADA8-4869-A16F-B9E7BC86E430}" name="diffusion_type" dataDxfId="29"/>
+    <tableColumn id="16" xr3:uid="{A99CC35E-FB67-451C-BF9C-DA8D933B1B0C}" name="multiplier" dataDxfId="28">
       <calculatedColumnFormula array="1">_xlfn.SWITCH(data[[#This Row],[diffusion_type]],"lognormal",0.0001,"normal",-0.01)*IF(data[[#This Row],[asset_class]]="Vol",1,1)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="8" xr3:uid="{02943B27-7FCB-4450-B8E0-CF0DB6CF5CCA}" name="factor_name_new" dataDxfId="38"/>
-    <tableColumn id="4" xr3:uid="{D181BF84-863F-4FD0-B518-14EA5B0FB18E}" name="description_override" dataDxfId="37"/>
-    <tableColumn id="6" xr3:uid="{1C40DF9B-2910-4DE6-A188-563938E39797}" name="Description_GPT" dataDxfId="36"/>
-    <tableColumn id="5" xr3:uid="{1806E074-6CB5-47AB-8FA3-EF0F6E429062}" name="Underlying" dataDxfId="35"/>
-    <tableColumn id="7" xr3:uid="{21539C17-C1CC-4FA9-A0E1-A2F8FF8AB52C}" name="Active" dataDxfId="34"/>
-    <tableColumn id="37" xr3:uid="{DE50B7AE-5F67-471C-BE48-8BFA5076EDB0}" name="hyper_factor" dataDxfId="33"/>
-    <tableColumn id="10" xr3:uid="{494805E4-EBB6-47FD-9BC2-8DAD9FB9D3FA}" name="composite" dataDxfId="32"/>
-    <tableColumn id="14" xr3:uid="{608FE572-4016-436E-8625-08926F3A2371}" name="client" dataDxfId="31"/>
-    <tableColumn id="13" xr3:uid="{64EF0381-B0C5-4226-B34E-0F9752A4A840}" name="ticker" dataDxfId="30">
+    <tableColumn id="8" xr3:uid="{02943B27-7FCB-4450-B8E0-CF0DB6CF5CCA}" name="factor_name_new" dataDxfId="27"/>
+    <tableColumn id="4" xr3:uid="{D181BF84-863F-4FD0-B518-14EA5B0FB18E}" name="description_override" dataDxfId="26"/>
+    <tableColumn id="6" xr3:uid="{1C40DF9B-2910-4DE6-A188-563938E39797}" name="Description_GPT" dataDxfId="25"/>
+    <tableColumn id="5" xr3:uid="{1806E074-6CB5-47AB-8FA3-EF0F6E429062}" name="Underlying" dataDxfId="24"/>
+    <tableColumn id="7" xr3:uid="{21539C17-C1CC-4FA9-A0E1-A2F8FF8AB52C}" name="Active" dataDxfId="23"/>
+    <tableColumn id="37" xr3:uid="{DE50B7AE-5F67-471C-BE48-8BFA5076EDB0}" name="hyper_factor" dataDxfId="22"/>
+    <tableColumn id="10" xr3:uid="{494805E4-EBB6-47FD-9BC2-8DAD9FB9D3FA}" name="composite" dataDxfId="21"/>
+    <tableColumn id="14" xr3:uid="{608FE572-4016-436E-8625-08926F3A2371}" name="client" dataDxfId="20"/>
+    <tableColumn id="13" xr3:uid="{64EF0381-B0C5-4226-B34E-0F9752A4A840}" name="ticker" dataDxfId="19">
       <calculatedColumnFormula>data[[#This Row],[factor_name]]</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="9" xr3:uid="{5A601067-D384-419C-A711-AD3034F77E28}" name="description" dataDxfId="29">
+    <tableColumn id="9" xr3:uid="{5A601067-D384-419C-A711-AD3034F77E28}" name="description" dataDxfId="18">
       <calculatedColumnFormula array="1">_xlfn.IFS(data[[#This Row],[description_override]]&lt;&gt;"",data[[#This Row],[description_override]],data[[#This Row],[Description_GPT]]&lt;&gt;"",data[[#This Row],[Description_GPT]],data[[#This Row],[Underlying]]&lt;&gt;"",data[[#This Row],[Underlying]],TRUE,"-")</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="18" xr3:uid="{073BDADC-3AC0-4FF9-9654-A316B2345A90}" name="short_name_yf" dataDxfId="28">
+    <tableColumn id="18" xr3:uid="{073BDADC-3AC0-4FF9-9654-A316B2345A90}" name="short_name_yf" dataDxfId="17">
       <calculatedColumnFormula>_xlfn.XLOOKUP(data[[#This Row],[ticker]],yf_desc[ticker],yf_desc[shortName],"-")</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="19" xr3:uid="{3A563104-B6B0-465C-9D22-154F5FEA1B83}" name="long_name_yf" dataDxfId="27">
+    <tableColumn id="19" xr3:uid="{3A563104-B6B0-465C-9D22-154F5FEA1B83}" name="long_name_yf" dataDxfId="16">
       <calculatedColumnFormula>_xlfn.XLOOKUP(data[[#This Row],[ticker]],yf_desc[ticker],yf_desc[longName],"-")</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="17" xr3:uid="{A3F200A1-E769-49BA-8121-88EAA1180E80}" name="summary_yf" dataDxfId="26">
+    <tableColumn id="17" xr3:uid="{A3F200A1-E769-49BA-8121-88EAA1180E80}" name="summary_yf" dataDxfId="15">
       <calculatedColumnFormula>_xlfn.XLOOKUP(data[[#This Row],[ticker]],yf_desc[ticker],yf_desc[longBusinessSummary],"-")</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="15" xr3:uid="{D49341AB-DA48-473E-8CCB-3A3D04AED743}" name="note" dataDxfId="25"/>
+    <tableColumn id="15" xr3:uid="{D49341AB-DA48-473E-8CCB-3A3D04AED743}" name="note" dataDxfId="14"/>
   </tableColumns>
   <tableStyleInfo name="Table Style 1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{F918301C-859F-40B7-9C3E-90E8F0495E68}" name="data_old" displayName="data_old" ref="A1:I45" totalsRowShown="0" headerRowDxfId="24" dataDxfId="23">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{F918301C-859F-40B7-9C3E-90E8F0495E68}" name="data_old" displayName="data_old" ref="A1:I45" totalsRowShown="0" headerRowDxfId="13" dataDxfId="12">
   <autoFilter ref="A1:I45" xr:uid="{6DAD1482-C63D-400D-9F51-F22A8E35CAD8}"/>
   <tableColumns count="9">
-    <tableColumn id="1" xr3:uid="{B19D2B17-9AC9-4F1B-B32E-D4F72AAE469F}" name="asset_class" dataDxfId="22"/>
-    <tableColumn id="2" xr3:uid="{2C7CF29D-8E72-4B0C-A212-31F2A25D75C9}" name="region" dataDxfId="21"/>
-    <tableColumn id="3" xr3:uid="{C7E89EEC-2B5D-4C94-9327-1AC8E33DE708}" name="factor_name" dataDxfId="20"/>
-    <tableColumn id="8" xr3:uid="{B3F9004A-8BEB-463E-A746-8189A2AC2B3E}" name="factor_name_new" dataDxfId="19"/>
-    <tableColumn id="4" xr3:uid="{51CD7FB3-58FE-4906-B73C-7726C0A9C471}" name="description_override" dataDxfId="18"/>
-    <tableColumn id="6" xr3:uid="{3CFF990B-3164-4533-821F-08CE7C6D82CA}" name="Description_GPT" dataDxfId="17"/>
-    <tableColumn id="5" xr3:uid="{DD86D53E-A9B4-4387-ABF9-F2625E77982D}" name="Underlying" dataDxfId="16"/>
-    <tableColumn id="7" xr3:uid="{D56FFF9A-72FF-42A4-B3D2-2F27AB16AF7A}" name="Active" dataDxfId="15"/>
-    <tableColumn id="9" xr3:uid="{8476DFDE-B4B1-4FD9-99B4-DF1F2ABBD7D5}" name="description" dataDxfId="14">
+    <tableColumn id="1" xr3:uid="{B19D2B17-9AC9-4F1B-B32E-D4F72AAE469F}" name="asset_class" dataDxfId="11"/>
+    <tableColumn id="2" xr3:uid="{2C7CF29D-8E72-4B0C-A212-31F2A25D75C9}" name="region" dataDxfId="10"/>
+    <tableColumn id="3" xr3:uid="{C7E89EEC-2B5D-4C94-9327-1AC8E33DE708}" name="factor_name" dataDxfId="9"/>
+    <tableColumn id="8" xr3:uid="{B3F9004A-8BEB-463E-A746-8189A2AC2B3E}" name="factor_name_new" dataDxfId="8"/>
+    <tableColumn id="4" xr3:uid="{51CD7FB3-58FE-4906-B73C-7726C0A9C471}" name="description_override" dataDxfId="7"/>
+    <tableColumn id="6" xr3:uid="{3CFF990B-3164-4533-821F-08CE7C6D82CA}" name="Description_GPT" dataDxfId="6"/>
+    <tableColumn id="5" xr3:uid="{DD86D53E-A9B4-4387-ABF9-F2625E77982D}" name="Underlying" dataDxfId="5"/>
+    <tableColumn id="7" xr3:uid="{D56FFF9A-72FF-42A4-B3D2-2F27AB16AF7A}" name="Active" dataDxfId="4"/>
+    <tableColumn id="9" xr3:uid="{8476DFDE-B4B1-4FD9-99B4-DF1F2ABBD7D5}" name="description" dataDxfId="3">
       <calculatedColumnFormula>IF(data_old[[#This Row],[description_override]]="",data_old[[#This Row],[Description_GPT]],data_old[[#This Row],[description_override]])</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -5792,11 +5720,12 @@
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3C29859C-7358-4E2F-B5CC-7696F1DAC449}">
   <sheetPr codeName="Sheet7"/>
-  <dimension ref="A1:Y107"/>
+  <dimension ref="A1:Y106"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12.28515625" customWidth="1"/>
     <col min="2" max="2" width="8.42578125" customWidth="1"/>
+    <col min="3" max="3" width="13.28515625" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="18.42578125" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="44.28515625" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="59.140625" bestFit="1" customWidth="1"/>
@@ -12203,60 +12132,57 @@
     </row>
     <row r="104" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A104" s="4" t="s">
-        <v>444</v>
+        <v>527</v>
       </c>
       <c r="B104" s="4" t="s">
         <v>40</v>
       </c>
       <c r="C104" s="4" t="s">
-        <v>500</v>
+        <v>528</v>
       </c>
       <c r="D104" s="4" t="s">
-        <v>445</v>
+        <v>529</v>
       </c>
       <c r="E104" s="4" t="s">
-        <v>454</v>
-      </c>
-      <c r="F104" s="4" cm="1">
-        <f t="array" ref="F104">_xlfn.SWITCH(data[[#This Row],[diffusion_type]],"lognormal",0.0001,"normal",-0.01)*IF(data[[#This Row],[asset_class]]="Vol",1,1)</f>
-        <v>1E-4</v>
+        <v>467</v>
+      </c>
+      <c r="F104" s="4">
+        <v>0.01</v>
       </c>
       <c r="G104" s="4"/>
       <c r="H104" s="4"/>
       <c r="I104" s="4"/>
-      <c r="J104" s="4" t="str" cm="1">
-        <f t="array" ref="J104">_xlfn.XLOOKUP(data[[#This Row],[factor_name]],_xlfn.ANCHORARRAY(composites!$F$2),_xlfn.ANCHORARRAY(composites!$G$2))</f>
-        <v>GLD 0.21, FXY 0.30, FXF 0.37, ^VIX3M -0.04, XLP 0.15, XLY -0.15</v>
+      <c r="J104" s="4" t="s">
+        <v>530</v>
       </c>
       <c r="K104" s="4">
         <v>1</v>
       </c>
       <c r="L104" s="4">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M104" s="4">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N104" s="4">
         <v>0</v>
       </c>
-      <c r="O104" s="4" t="str">
-        <f>data[[#This Row],[factor_name]]</f>
-        <v>TRADEWAR</v>
+      <c r="O104" s="11" t="s">
+        <v>531</v>
       </c>
       <c r="P104" s="4" t="str" cm="1">
         <f t="array" ref="P104">_xlfn.IFS(data[[#This Row],[description_override]]&lt;&gt;"",data[[#This Row],[description_override]],data[[#This Row],[Description_GPT]]&lt;&gt;"",data[[#This Row],[Description_GPT]],data[[#This Row],[Underlying]]&lt;&gt;"",data[[#This Row],[Underlying]],TRUE,"-")</f>
-        <v>GLD 0.21, FXY 0.30, FXF 0.37, ^VIX3M -0.04, XLP 0.15, XLY -0.15</v>
-      </c>
-      <c r="Q104" s="4" t="str">
+        <v>Economic Policy Uncertainty Index for United States</v>
+      </c>
+      <c r="Q104" s="11" t="str">
         <f>_xlfn.XLOOKUP(data[[#This Row],[ticker]],yf_desc[ticker],yf_desc[shortName],"-")</f>
         <v>-</v>
       </c>
-      <c r="R104" s="4" t="str">
+      <c r="R104" s="11" t="str">
         <f>_xlfn.XLOOKUP(data[[#This Row],[ticker]],yf_desc[ticker],yf_desc[longName],"-")</f>
         <v>-</v>
       </c>
-      <c r="S104" s="4" t="str">
+      <c r="S104" s="11" t="str">
         <f>_xlfn.XLOOKUP(data[[#This Row],[ticker]],yf_desc[ticker],yf_desc[longBusinessSummary],"-")</f>
         <v>-</v>
       </c>
@@ -12264,29 +12190,28 @@
     </row>
     <row r="105" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A105" s="4" t="s">
-        <v>527</v>
+        <v>65</v>
       </c>
       <c r="B105" s="4" t="s">
         <v>40</v>
       </c>
       <c r="C105" s="4" t="s">
-        <v>528</v>
+        <v>682</v>
       </c>
       <c r="D105" s="4" t="s">
-        <v>529</v>
+        <v>686</v>
       </c>
       <c r="E105" s="4" t="s">
-        <v>467</v>
-      </c>
-      <c r="F105" s="4">
-        <v>0.01</v>
+        <v>454</v>
+      </c>
+      <c r="F105" s="4" cm="1">
+        <f t="array" ref="F105">_xlfn.SWITCH(data[[#This Row],[diffusion_type]],"lognormal",0.0001,"normal",-0.01)*IF(data[[#This Row],[asset_class]]="Vol",1,1)</f>
+        <v>1E-4</v>
       </c>
       <c r="G105" s="4"/>
       <c r="H105" s="4"/>
       <c r="I105" s="4"/>
-      <c r="J105" s="4" t="s">
-        <v>530</v>
-      </c>
+      <c r="J105" s="4"/>
       <c r="K105" s="4">
         <v>1</v>
       </c>
@@ -12299,22 +12224,22 @@
       <c r="N105" s="4">
         <v>0</v>
       </c>
-      <c r="O105" s="11" t="s">
-        <v>531</v>
+      <c r="O105" s="4" t="s">
+        <v>684</v>
       </c>
       <c r="P105" s="4" t="str" cm="1">
         <f t="array" ref="P105">_xlfn.IFS(data[[#This Row],[description_override]]&lt;&gt;"",data[[#This Row],[description_override]],data[[#This Row],[Description_GPT]]&lt;&gt;"",data[[#This Row],[Description_GPT]],data[[#This Row],[Underlying]]&lt;&gt;"",data[[#This Row],[Underlying]],TRUE,"-")</f>
-        <v>Economic Policy Uncertainty Index for United States</v>
-      </c>
-      <c r="Q105" s="11" t="str">
+        <v>-</v>
+      </c>
+      <c r="Q105" s="4" t="str">
         <f>_xlfn.XLOOKUP(data[[#This Row],[ticker]],yf_desc[ticker],yf_desc[shortName],"-")</f>
         <v>-</v>
       </c>
-      <c r="R105" s="11" t="str">
+      <c r="R105" s="4" t="str">
         <f>_xlfn.XLOOKUP(data[[#This Row],[ticker]],yf_desc[ticker],yf_desc[longName],"-")</f>
         <v>-</v>
       </c>
-      <c r="S105" s="11" t="str">
+      <c r="S105" s="4" t="str">
         <f>_xlfn.XLOOKUP(data[[#This Row],[ticker]],yf_desc[ticker],yf_desc[longBusinessSummary],"-")</f>
         <v>-</v>
       </c>
@@ -12322,23 +12247,23 @@
     </row>
     <row r="106" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A106" s="4" t="s">
-        <v>65</v>
+        <v>475</v>
       </c>
       <c r="B106" s="4" t="s">
         <v>40</v>
       </c>
       <c r="C106" s="4" t="s">
-        <v>682</v>
+        <v>683</v>
       </c>
       <c r="D106" s="4" t="s">
         <v>686</v>
       </c>
       <c r="E106" s="4" t="s">
-        <v>454</v>
+        <v>467</v>
       </c>
       <c r="F106" s="4" cm="1">
         <f t="array" ref="F106">_xlfn.SWITCH(data[[#This Row],[diffusion_type]],"lognormal",0.0001,"normal",-0.01)*IF(data[[#This Row],[asset_class]]="Vol",1,1)</f>
-        <v>1E-4</v>
+        <v>-0.01</v>
       </c>
       <c r="G106" s="4"/>
       <c r="H106" s="4"/>
@@ -12357,7 +12282,7 @@
         <v>0</v>
       </c>
       <c r="O106" s="4" t="s">
-        <v>684</v>
+        <v>685</v>
       </c>
       <c r="P106" s="4" t="str" cm="1">
         <f t="array" ref="P106">_xlfn.IFS(data[[#This Row],[description_override]]&lt;&gt;"",data[[#This Row],[description_override]],data[[#This Row],[Description_GPT]]&lt;&gt;"",data[[#This Row],[Description_GPT]],data[[#This Row],[Underlying]]&lt;&gt;"",data[[#This Row],[Underlying]],TRUE,"-")</f>
@@ -12376,63 +12301,6 @@
         <v>-</v>
       </c>
       <c r="T106" s="4"/>
-    </row>
-    <row r="107" spans="1:20" x14ac:dyDescent="0.25">
-      <c r="A107" s="4" t="s">
-        <v>475</v>
-      </c>
-      <c r="B107" s="4" t="s">
-        <v>40</v>
-      </c>
-      <c r="C107" s="4" t="s">
-        <v>683</v>
-      </c>
-      <c r="D107" s="4" t="s">
-        <v>686</v>
-      </c>
-      <c r="E107" s="4" t="s">
-        <v>467</v>
-      </c>
-      <c r="F107" s="4" cm="1">
-        <f t="array" ref="F107">_xlfn.SWITCH(data[[#This Row],[diffusion_type]],"lognormal",0.0001,"normal",-0.01)*IF(data[[#This Row],[asset_class]]="Vol",1,1)</f>
-        <v>-0.01</v>
-      </c>
-      <c r="G107" s="4"/>
-      <c r="H107" s="4"/>
-      <c r="I107" s="4"/>
-      <c r="J107" s="4"/>
-      <c r="K107" s="4">
-        <v>1</v>
-      </c>
-      <c r="L107" s="4">
-        <v>0</v>
-      </c>
-      <c r="M107" s="4">
-        <v>0</v>
-      </c>
-      <c r="N107" s="4">
-        <v>0</v>
-      </c>
-      <c r="O107" s="4" t="s">
-        <v>685</v>
-      </c>
-      <c r="P107" s="4" t="str" cm="1">
-        <f t="array" ref="P107">_xlfn.IFS(data[[#This Row],[description_override]]&lt;&gt;"",data[[#This Row],[description_override]],data[[#This Row],[Description_GPT]]&lt;&gt;"",data[[#This Row],[Description_GPT]],data[[#This Row],[Underlying]]&lt;&gt;"",data[[#This Row],[Underlying]],TRUE,"-")</f>
-        <v>-</v>
-      </c>
-      <c r="Q107" s="4" t="str">
-        <f>_xlfn.XLOOKUP(data[[#This Row],[ticker]],yf_desc[ticker],yf_desc[shortName],"-")</f>
-        <v>-</v>
-      </c>
-      <c r="R107" s="4" t="str">
-        <f>_xlfn.XLOOKUP(data[[#This Row],[ticker]],yf_desc[ticker],yf_desc[longName],"-")</f>
-        <v>-</v>
-      </c>
-      <c r="S107" s="4" t="str">
-        <f>_xlfn.XLOOKUP(data[[#This Row],[ticker]],yf_desc[ticker],yf_desc[longBusinessSummary],"-")</f>
-        <v>-</v>
-      </c>
-      <c r="T107" s="4"/>
     </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>
@@ -12612,7 +12480,7 @@
 
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E5A64DEF-E706-4B9C-B282-71F34F86B3DF}">
-  <dimension ref="A1:J87"/>
+  <dimension ref="A1:J86"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="6" max="6" width="44.28515625" bestFit="1" customWidth="1"/>
@@ -12652,11 +12520,11 @@
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2" t="str" cm="1">
-        <f t="array" ref="A2:A87">_xlfn._xlws.FILTER(data[factor_name],data[Active])</f>
+        <f t="array" ref="A2:A86">_xlfn._xlws.FILTER(data[factor_name],data[Active])</f>
         <v>SPY</v>
       </c>
       <c r="B2" t="str" cm="1">
-        <f t="array" ref="B2:J87">INDEX(data[],_xlfn.XMATCH(_xlfn.ANCHORARRAY(A2),data[factor_name]),_xlfn.XMATCH(B1:J1,data[#Headers]))</f>
+        <f t="array" ref="B2:J86">INDEX(data[],_xlfn.XMATCH(_xlfn.ANCHORARRAY(A2),data[factor_name]),_xlfn.XMATCH(B1:J1,data[#Headers]))</f>
         <v>Equities</v>
       </c>
       <c r="C2" t="str">
@@ -15278,42 +15146,42 @@
     </row>
     <row r="84" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A84" t="str">
-        <v>TRADEWAR</v>
+        <v>UNCERTAINTY</v>
       </c>
       <c r="B84" t="str">
-        <v>Theme</v>
+        <v>Econ</v>
       </c>
       <c r="C84" t="str">
         <v>USD</v>
       </c>
       <c r="D84">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E84">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F84" t="str">
-        <v>GLD 0.21, FXY 0.30, FXF 0.37, ^VIX3M -0.04, XLP 0.15, XLY -0.15</v>
+        <v>Economic Policy Uncertainty Index for United States</v>
       </c>
       <c r="G84" t="str">
-        <v>composite</v>
+        <v>fred</v>
       </c>
       <c r="H84" t="str">
-        <v>TRADEWAR</v>
+        <v>USEPUINDXD</v>
       </c>
       <c r="I84" t="str">
-        <v>lognormal</v>
+        <v>normal</v>
       </c>
       <c r="J84">
-        <v>1E-4</v>
+        <v>0.01</v>
       </c>
     </row>
     <row r="85" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A85" t="str">
-        <v>UNCERTAINTY</v>
+        <v>BTC</v>
       </c>
       <c r="B85" t="str">
-        <v>Econ</v>
+        <v>Currencies</v>
       </c>
       <c r="C85" t="str">
         <v>USD</v>
@@ -15325,27 +15193,27 @@
         <v>0</v>
       </c>
       <c r="F85" t="str">
-        <v>Economic Policy Uncertainty Index for United States</v>
+        <v>-</v>
       </c>
       <c r="G85" t="str">
-        <v>fred</v>
+        <v>lmxl</v>
       </c>
       <c r="H85" t="str">
-        <v>USEPUINDXD</v>
+        <v>BTC1_price</v>
       </c>
       <c r="I85" t="str">
-        <v>normal</v>
+        <v>lognormal</v>
       </c>
       <c r="J85">
-        <v>0.01</v>
+        <v>1E-4</v>
       </c>
     </row>
     <row r="86" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A86" t="str">
-        <v>BTC</v>
+        <v>BTC_vol</v>
       </c>
       <c r="B86" t="str">
-        <v>Currencies</v>
+        <v>Vol</v>
       </c>
       <c r="C86" t="str">
         <v>USD</v>
@@ -15363,44 +15231,12 @@
         <v>lmxl</v>
       </c>
       <c r="H86" t="str">
-        <v>BTC1_price</v>
+        <v>BTC1_atm</v>
       </c>
       <c r="I86" t="str">
-        <v>lognormal</v>
+        <v>normal</v>
       </c>
       <c r="J86">
-        <v>1E-4</v>
-      </c>
-    </row>
-    <row r="87" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A87" t="str">
-        <v>BTC_vol</v>
-      </c>
-      <c r="B87" t="str">
-        <v>Vol</v>
-      </c>
-      <c r="C87" t="str">
-        <v>USD</v>
-      </c>
-      <c r="D87">
-        <v>0</v>
-      </c>
-      <c r="E87">
-        <v>0</v>
-      </c>
-      <c r="F87" t="str">
-        <v>-</v>
-      </c>
-      <c r="G87" t="str">
-        <v>lmxl</v>
-      </c>
-      <c r="H87" t="str">
-        <v>BTC1_atm</v>
-      </c>
-      <c r="I87" t="str">
-        <v>normal</v>
-      </c>
-      <c r="J87">
         <v>-0.01</v>
       </c>
     </row>
@@ -17795,7 +17631,7 @@
 <file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2977BD7F-9323-4F6D-98BF-C1B39119DCDE}">
   <sheetPr codeName="Sheet8"/>
-  <dimension ref="A1:J87"/>
+  <dimension ref="A1:J86"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="6" max="6" width="44.28515625" bestFit="1" customWidth="1"/>
@@ -17835,11 +17671,11 @@
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2" t="str" cm="1">
-        <f t="array" ref="A2:A87">_xlfn._xlws.FILTER(data[factor_name],data[Active]*(data[client]=0))</f>
+        <f t="array" ref="A2:A86">_xlfn._xlws.FILTER(data[factor_name],data[Active]*(data[client]=0))</f>
         <v>SPY</v>
       </c>
       <c r="B2" t="str" cm="1">
-        <f t="array" ref="B2:J87">INDEX(data[],_xlfn.XMATCH(_xlfn.ANCHORARRAY(A2),data[factor_name]),_xlfn.XMATCH(B1:J1,data[#Headers]))</f>
+        <f t="array" ref="B2:J86">INDEX(data[],_xlfn.XMATCH(_xlfn.ANCHORARRAY(A2),data[factor_name]),_xlfn.XMATCH(B1:J1,data[#Headers]))</f>
         <v>Equities</v>
       </c>
       <c r="C2" t="str">
@@ -20461,42 +20297,42 @@
     </row>
     <row r="84" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A84" t="str">
-        <v>TRADEWAR</v>
+        <v>UNCERTAINTY</v>
       </c>
       <c r="B84" t="str">
-        <v>Theme</v>
+        <v>Econ</v>
       </c>
       <c r="C84" t="str">
         <v>USD</v>
       </c>
       <c r="D84">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E84">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F84" t="str">
-        <v>GLD 0.21, FXY 0.30, FXF 0.37, ^VIX3M -0.04, XLP 0.15, XLY -0.15</v>
+        <v>Economic Policy Uncertainty Index for United States</v>
       </c>
       <c r="G84" t="str">
-        <v>composite</v>
+        <v>fred</v>
       </c>
       <c r="H84" t="str">
-        <v>TRADEWAR</v>
+        <v>USEPUINDXD</v>
       </c>
       <c r="I84" t="str">
-        <v>lognormal</v>
+        <v>normal</v>
       </c>
       <c r="J84">
-        <v>1E-4</v>
+        <v>0.01</v>
       </c>
     </row>
     <row r="85" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A85" t="str">
-        <v>UNCERTAINTY</v>
+        <v>BTC</v>
       </c>
       <c r="B85" t="str">
-        <v>Econ</v>
+        <v>Currencies</v>
       </c>
       <c r="C85" t="str">
         <v>USD</v>
@@ -20508,27 +20344,27 @@
         <v>0</v>
       </c>
       <c r="F85" t="str">
-        <v>Economic Policy Uncertainty Index for United States</v>
+        <v>-</v>
       </c>
       <c r="G85" t="str">
-        <v>fred</v>
+        <v>lmxl</v>
       </c>
       <c r="H85" t="str">
-        <v>USEPUINDXD</v>
+        <v>BTC1_price</v>
       </c>
       <c r="I85" t="str">
-        <v>normal</v>
+        <v>lognormal</v>
       </c>
       <c r="J85">
-        <v>0.01</v>
+        <v>1E-4</v>
       </c>
     </row>
     <row r="86" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A86" t="str">
-        <v>BTC</v>
+        <v>BTC_vol</v>
       </c>
       <c r="B86" t="str">
-        <v>Currencies</v>
+        <v>Vol</v>
       </c>
       <c r="C86" t="str">
         <v>USD</v>
@@ -20546,44 +20382,12 @@
         <v>lmxl</v>
       </c>
       <c r="H86" t="str">
-        <v>BTC1_price</v>
+        <v>BTC1_atm</v>
       </c>
       <c r="I86" t="str">
-        <v>lognormal</v>
+        <v>normal</v>
       </c>
       <c r="J86">
-        <v>1E-4</v>
-      </c>
-    </row>
-    <row r="87" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A87" t="str">
-        <v>BTC_vol</v>
-      </c>
-      <c r="B87" t="str">
-        <v>Vol</v>
-      </c>
-      <c r="C87" t="str">
-        <v>USD</v>
-      </c>
-      <c r="D87">
-        <v>0</v>
-      </c>
-      <c r="E87">
-        <v>0</v>
-      </c>
-      <c r="F87" t="str">
-        <v>-</v>
-      </c>
-      <c r="G87" t="str">
-        <v>lmxl</v>
-      </c>
-      <c r="H87" t="str">
-        <v>BTC1_atm</v>
-      </c>
-      <c r="I87" t="str">
-        <v>normal</v>
-      </c>
-      <c r="J87">
         <v>-0.01</v>
       </c>
     </row>

</xml_diff>

<commit_message>
data: Update the SOFTWARE-SEMI factor to make it beta 1 to QQQ
</commit_message>
<xml_diff>
--- a/factor_master.xlsx
+++ b/factor_master.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\bkrai\Source\risk\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F9BBBDC7-40CE-4F2B-ABE0-9F9DDC1790A2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D1B54171-EAE9-4306-B460-2C14ECFCA98B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" firstSheet="8" activeTab="10" xr2:uid="{C31FDC5B-A809-4BFD-99CB-DA02246721F7}"/>
   </bookViews>
@@ -103,7 +103,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2589" uniqueCount="728">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2592" uniqueCount="729">
   <si>
     <t>SPX</t>
   </si>
@@ -2287,6 +2287,9 @@
   </si>
   <si>
     <t>PRIVATES</t>
+  </si>
+  <si>
+    <t>x</t>
   </si>
 </sst>
 </file>
@@ -2810,8 +2813,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{B096ECD9-9D11-4532-B7BB-C59C7AF13EE1}" name="composities" displayName="composities" ref="A1:C27" totalsRowShown="0">
-  <autoFilter ref="A1:C27" xr:uid="{B096ECD9-9D11-4532-B7BB-C59C7AF13EE1}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{B096ECD9-9D11-4532-B7BB-C59C7AF13EE1}" name="composities" displayName="composities" ref="A1:C28" totalsRowShown="0">
+  <autoFilter ref="A1:C28" xr:uid="{B096ECD9-9D11-4532-B7BB-C59C7AF13EE1}"/>
   <tableColumns count="3">
     <tableColumn id="1" xr3:uid="{871951C6-7319-4AA1-8565-79E8F38A5ACE}" name="portfolio_name"/>
     <tableColumn id="2" xr3:uid="{FF366C7B-7C4B-413F-92EE-C488EBE75CC9}" name="factor_name"/>
@@ -4793,7 +4796,7 @@
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{75C34FC6-78FE-492E-BECF-2EB9A04778A9}">
   <sheetPr codeName="Sheet6"/>
-  <dimension ref="A1:AJ40"/>
+  <dimension ref="A1:AJ41"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="15.42578125" customWidth="1"/>
@@ -4833,11 +4836,11 @@
         <v>1</v>
       </c>
       <c r="E2" s="23" cm="1">
-        <f t="array" ref="E2:E27">_xlfn.XLOOKUP(composities[portfolio_name],data[factor_name],data[Active])</f>
+        <f t="array" ref="E2:E28">_xlfn.XLOOKUP(composities[portfolio_name],data[factor_name],data[Active])</f>
         <v>1</v>
       </c>
       <c r="H2" t="str" cm="1">
-        <f t="array" ref="H2:H27">TEXT(composities[weight],IF(INT(composities[weight]*100)/100=composities[weight],"General","0.00"))</f>
+        <f t="array" ref="H2:H28">TEXT(composities[weight],IF(INT(composities[weight]*100)/100=composities[weight],"General","0.00"))</f>
         <v>1</v>
       </c>
       <c r="I2" t="str" cm="1">
@@ -4849,7 +4852,7 @@
         <v>SHY 1, BSV 1</v>
       </c>
       <c r="X2" t="b" cm="1">
-        <f t="array" aca="1" ref="X2:X27" ca="1">composities[portfolio_name]&lt;&gt;OFFSET(composities[portfolio_name],-1,0)</f>
+        <f t="array" aca="1" ref="X2:X28" ca="1">composities[portfolio_name]&lt;&gt;OFFSET(composities[portfolio_name],-1,0)</f>
         <v>1</v>
       </c>
       <c r="AE2" t="s">
@@ -5113,7 +5116,7 @@
         <v>SEMI-SOFT</v>
       </c>
       <c r="J9" t="str">
-        <v>SMH 1, IGV -1</v>
+        <v>SMH 1, IGV -1, QQQ 1</v>
       </c>
       <c r="X9" t="b">
         <f ca="1"/>
@@ -5144,6 +5147,9 @@
       </c>
       <c r="E10" s="23">
         <v>1</v>
+      </c>
+      <c r="F10" s="23" t="s">
+        <v>728</v>
       </c>
       <c r="H10" t="str">
         <v>-0.05</v>
@@ -5603,23 +5609,23 @@
     </row>
     <row r="24" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>727</v>
+        <v>723</v>
       </c>
       <c r="B24" t="s">
-        <v>724</v>
+        <v>7</v>
       </c>
       <c r="C24" s="8">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="E24" s="23">
         <v>1</v>
       </c>
       <c r="H24" t="str">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="X24" t="b">
         <f ca="1"/>
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="25" spans="1:26" x14ac:dyDescent="0.25">
@@ -5627,20 +5633,20 @@
         <v>727</v>
       </c>
       <c r="B25" t="s">
-        <v>175</v>
+        <v>724</v>
       </c>
       <c r="C25" s="8">
-        <v>-0.5</v>
+        <v>0.5</v>
       </c>
       <c r="E25" s="23">
         <v>1</v>
       </c>
       <c r="H25" t="str">
-        <v>-0.5</v>
+        <v>0.5</v>
       </c>
       <c r="X25" t="b">
         <f ca="1"/>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="26" spans="1:26" x14ac:dyDescent="0.25">
@@ -5648,16 +5654,16 @@
         <v>727</v>
       </c>
       <c r="B26" t="s">
-        <v>293</v>
+        <v>175</v>
       </c>
       <c r="C26" s="8">
-        <v>0.5</v>
+        <v>-0.5</v>
       </c>
       <c r="E26" s="23">
         <v>1</v>
       </c>
       <c r="H26" t="str">
-        <v>0.5</v>
+        <v>-0.5</v>
       </c>
       <c r="X26" t="b">
         <f ca="1"/>
@@ -5669,16 +5675,16 @@
         <v>727</v>
       </c>
       <c r="B27" t="s">
-        <v>347</v>
+        <v>293</v>
       </c>
       <c r="C27" s="8">
-        <v>-0.5</v>
+        <v>0.5</v>
       </c>
       <c r="E27" s="23">
         <v>1</v>
       </c>
       <c r="H27" t="str">
-        <v>-0.5</v>
+        <v>0.5</v>
       </c>
       <c r="X27" t="b">
         <f ca="1"/>
@@ -5686,7 +5692,25 @@
       </c>
     </row>
     <row r="28" spans="1:26" x14ac:dyDescent="0.25">
-      <c r="C28" s="8"/>
+      <c r="A28" t="s">
+        <v>727</v>
+      </c>
+      <c r="B28" t="s">
+        <v>347</v>
+      </c>
+      <c r="C28" s="8">
+        <v>-0.5</v>
+      </c>
+      <c r="E28" s="23">
+        <v>1</v>
+      </c>
+      <c r="H28" t="str">
+        <v>-0.5</v>
+      </c>
+      <c r="X28" t="b">
+        <f ca="1"/>
+        <v>0</v>
+      </c>
     </row>
     <row r="29" spans="1:26" x14ac:dyDescent="0.25">
       <c r="C29" s="8"/>
@@ -5699,6 +5723,9 @@
     </row>
     <row r="32" spans="1:26" x14ac:dyDescent="0.25">
       <c r="C32" s="8"/>
+    </row>
+    <row r="33" spans="1:26" x14ac:dyDescent="0.25">
+      <c r="C33" s="8"/>
     </row>
     <row r="34" spans="1:26" x14ac:dyDescent="0.25">
       <c r="Q34" t="e" vm="1">
@@ -5737,21 +5764,11 @@
         <v>#VALUE!</v>
       </c>
       <c r="W36" cm="1">
-        <f t="array" ref="W36:W39">C37:C40*N36:N39</f>
+        <f t="array" ref="W36:W39">C38:C41*N36:N39</f>
         <v>3</v>
       </c>
     </row>
     <row r="37" spans="1:26" x14ac:dyDescent="0.25">
-      <c r="A37" t="s">
-        <v>504</v>
-      </c>
-      <c r="B37" t="s">
-        <v>57</v>
-      </c>
-      <c r="C37" s="8">
-        <f>O36/N36</f>
-        <v>0.20547945205479454</v>
-      </c>
       <c r="D37" s="8"/>
       <c r="G37" s="8"/>
       <c r="H37" s="8"/>
@@ -5781,11 +5798,11 @@
         <v>504</v>
       </c>
       <c r="B38" t="s">
-        <v>72</v>
+        <v>57</v>
       </c>
       <c r="C38" s="8">
-        <f>O37/N37</f>
-        <v>0.29702970297029702</v>
+        <f>O36/N36</f>
+        <v>0.20547945205479454</v>
       </c>
       <c r="D38" s="8"/>
       <c r="G38" s="8"/>
@@ -5813,11 +5830,11 @@
         <v>504</v>
       </c>
       <c r="B39" t="s">
-        <v>497</v>
+        <v>72</v>
       </c>
       <c r="C39" s="8">
-        <f>O38/N38</f>
-        <v>0.36585365853658541</v>
+        <f>O37/N37</f>
+        <v>0.29702970297029702</v>
       </c>
       <c r="D39" s="8"/>
       <c r="G39" s="8"/>
@@ -5843,9 +5860,21 @@
         <v>504</v>
       </c>
       <c r="B40" t="s">
+        <v>497</v>
+      </c>
+      <c r="C40" s="8">
+        <f>O38/N38</f>
+        <v>0.36585365853658541</v>
+      </c>
+    </row>
+    <row r="41" spans="1:26" x14ac:dyDescent="0.25">
+      <c r="A41" t="s">
+        <v>504</v>
+      </c>
+      <c r="B41" t="s">
         <v>495</v>
       </c>
-      <c r="C40" s="8">
+      <c r="C41" s="8">
         <f>O39/N39</f>
         <v>-0.1125</v>
       </c>
@@ -5856,22 +5885,22 @@
       <formula>$Q1048571</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A11:C18">
+  <conditionalFormatting sqref="A11:C18 A25:C28">
     <cfRule type="expression" dxfId="4" priority="41">
       <formula>$T6</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A19:C27">
+  <conditionalFormatting sqref="A19:C24">
     <cfRule type="expression" dxfId="3" priority="40">
       <formula>$T15</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A31:C32">
+  <conditionalFormatting sqref="A32:C33">
     <cfRule type="expression" dxfId="2" priority="42">
       <formula>$T19</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A28:C30">
+  <conditionalFormatting sqref="A29:C31">
     <cfRule type="expression" dxfId="1" priority="44">
       <formula>$T21</formula>
     </cfRule>
@@ -12197,7 +12226,7 @@
       <c r="I102" s="4"/>
       <c r="J102" s="4" t="str" cm="1">
         <f t="array" ref="J102">_xlfn.XLOOKUP(data[[#This Row],[factor_name]],_xlfn.ANCHORARRAY(composites!$I$2),_xlfn.ANCHORARRAY(composites!$J$2))</f>
-        <v>SMH 1, IGV -1</v>
+        <v>SMH 1, IGV -1, QQQ 1</v>
       </c>
       <c r="K102" s="4">
         <v>1</v>
@@ -12217,7 +12246,7 @@
       </c>
       <c r="P102" s="4" t="str" cm="1">
         <f t="array" ref="P102">_xlfn.IFS(data[[#This Row],[description_override]]&lt;&gt;"",data[[#This Row],[description_override]],data[[#This Row],[Description_GPT]]&lt;&gt;"",data[[#This Row],[Description_GPT]],data[[#This Row],[Underlying]]&lt;&gt;"",data[[#This Row],[Underlying]],TRUE,"-")</f>
-        <v>SMH 1, IGV -1</v>
+        <v>SMH 1, IGV -1, QQQ 1</v>
       </c>
       <c r="Q102" s="4" t="str">
         <f>_xlfn.XLOOKUP(data[[#This Row],[ticker]],yf_desc[ticker],yf_desc[shortName],"-")</f>
@@ -15309,7 +15338,7 @@
         <v>1</v>
       </c>
       <c r="F81" t="str">
-        <v>SMH 1, IGV -1</v>
+        <v>SMH 1, IGV -1, QQQ 1</v>
       </c>
       <c r="G81" t="str">
         <v>composite</v>
@@ -20460,7 +20489,7 @@
         <v>1</v>
       </c>
       <c r="F81" t="str">
-        <v>SMH 1, IGV -1</v>
+        <v>SMH 1, IGV -1, QQQ 1</v>
       </c>
       <c r="G81" t="str">
         <v>composite</v>
@@ -27344,7 +27373,7 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B7A5BD3C-985E-4AF9-B99B-18E2DCAB8A90}">
   <sheetPr codeName="Sheet5"/>
-  <dimension ref="A1:C27"/>
+  <dimension ref="A1:C28"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
@@ -27361,7 +27390,7 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="str" cm="1">
-        <f t="array" ref="A2:C27">composities[]</f>
+        <f t="array" ref="A2:C28">composities[]</f>
         <v>FED</v>
       </c>
       <c r="B2" t="str">
@@ -27604,13 +27633,13 @@
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A24" t="str">
-        <v>PRIVATES</v>
+        <v>SEMI-SOFT</v>
       </c>
       <c r="B24" t="str">
-        <v>PSP</v>
+        <v>QQQ</v>
       </c>
       <c r="C24">
-        <v>0.5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.25">
@@ -27618,10 +27647,10 @@
         <v>PRIVATES</v>
       </c>
       <c r="B25" t="str">
-        <v>XLF</v>
+        <v>PSP</v>
       </c>
       <c r="C25">
-        <v>-0.5</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.25">
@@ -27629,10 +27658,10 @@
         <v>PRIVATES</v>
       </c>
       <c r="B26" t="str">
-        <v>BKLN</v>
+        <v>XLF</v>
       </c>
       <c r="C26">
-        <v>0.5</v>
+        <v>-0.5</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.25">
@@ -27640,9 +27669,20 @@
         <v>PRIVATES</v>
       </c>
       <c r="B27" t="str">
+        <v>BKLN</v>
+      </c>
+      <c r="C27">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A28" t="str">
+        <v>PRIVATES</v>
+      </c>
+      <c r="B28" t="str">
         <v>LQDH</v>
       </c>
-      <c r="C27">
+      <c r="C28">
         <v>-0.5</v>
       </c>
     </row>
@@ -27863,7 +27903,7 @@
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="10">
         <f ca="1">TODAY()-1</f>
-        <v>46130</v>
+        <v>46131</v>
       </c>
       <c r="B2">
         <v>0.20547945205479451</v>

</xml_diff>

<commit_message>
fix: Deactivate FRED data after API stopped working
</commit_message>
<xml_diff>
--- a/factor_master.xlsx
+++ b/factor_master.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30208"/>
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\bkrai\Source\risk\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D1B54171-EAE9-4306-B460-2C14ECFCA98B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4D8F7DF1-93C2-43EB-82ED-923B3F7BF83C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" firstSheet="8" activeTab="10" xr2:uid="{C31FDC5B-A809-4BFD-99CB-DA02246721F7}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" firstSheet="11" activeTab="11" xr2:uid="{C31FDC5B-A809-4BFD-99CB-DA02246721F7}"/>
   </bookViews>
   <sheets>
     <sheet name="legacy" sheetId="5" r:id="rId1"/>
@@ -2434,7 +2434,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -2459,15 +2459,11 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
@@ -2482,7 +2478,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2549,16 +2544,6 @@
         </top>
         <vertical/>
         <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <border outline="0">
-        <bottom style="thin">
-          <color theme="0" tint="-0.24994659260841701"/>
-        </bottom>
       </border>
     </dxf>
     <dxf>
@@ -2680,6 +2665,16 @@
     </dxf>
     <dxf>
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <bottom style="thin">
+          <color theme="0" tint="-0.24994659260841701"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <border>
@@ -2825,58 +2820,58 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{6DAD1482-C63D-400D-9F51-F22A8E35CAD8}" name="data" displayName="data" ref="A1:T107" totalsRowShown="0" headerRowDxfId="7" dataDxfId="40" headerRowBorderDxfId="8">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{6DAD1482-C63D-400D-9F51-F22A8E35CAD8}" name="data" displayName="data" ref="A1:T107" totalsRowShown="0" headerRowDxfId="40" dataDxfId="38" headerRowBorderDxfId="39">
   <tableColumns count="20">
-    <tableColumn id="1" xr3:uid="{740DC173-AAC9-4239-A44E-C43F8517304D}" name="asset_class" dataDxfId="39"/>
-    <tableColumn id="2" xr3:uid="{A3BC3BB8-0420-458E-AECD-FD567519FA40}" name="region" dataDxfId="38"/>
-    <tableColumn id="3" xr3:uid="{0E50B2E3-0362-41DB-ACC2-478CC6F618A4}" name="factor_name" dataDxfId="37"/>
-    <tableColumn id="11" xr3:uid="{C400A641-F032-4829-A2CD-62831D657B37}" name="source" dataDxfId="36"/>
-    <tableColumn id="12" xr3:uid="{BC682952-ADA8-4869-A16F-B9E7BC86E430}" name="diffusion_type" dataDxfId="35"/>
-    <tableColumn id="16" xr3:uid="{A99CC35E-FB67-451C-BF9C-DA8D933B1B0C}" name="multiplier" dataDxfId="34">
+    <tableColumn id="1" xr3:uid="{740DC173-AAC9-4239-A44E-C43F8517304D}" name="asset_class" dataDxfId="37"/>
+    <tableColumn id="2" xr3:uid="{A3BC3BB8-0420-458E-AECD-FD567519FA40}" name="region" dataDxfId="36"/>
+    <tableColumn id="3" xr3:uid="{0E50B2E3-0362-41DB-ACC2-478CC6F618A4}" name="factor_name" dataDxfId="35"/>
+    <tableColumn id="11" xr3:uid="{C400A641-F032-4829-A2CD-62831D657B37}" name="source" dataDxfId="34"/>
+    <tableColumn id="12" xr3:uid="{BC682952-ADA8-4869-A16F-B9E7BC86E430}" name="diffusion_type" dataDxfId="33"/>
+    <tableColumn id="16" xr3:uid="{A99CC35E-FB67-451C-BF9C-DA8D933B1B0C}" name="multiplier" dataDxfId="32">
       <calculatedColumnFormula array="1">_xlfn.SWITCH(data[[#This Row],[diffusion_type]],"lognormal",0.0001,"normal",-0.01)*IF(data[[#This Row],[asset_class]]="Vol",1,1)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="8" xr3:uid="{02943B27-7FCB-4450-B8E0-CF0DB6CF5CCA}" name="factor_name_new" dataDxfId="33"/>
-    <tableColumn id="4" xr3:uid="{D181BF84-863F-4FD0-B518-14EA5B0FB18E}" name="description_override" dataDxfId="32"/>
-    <tableColumn id="6" xr3:uid="{1C40DF9B-2910-4DE6-A188-563938E39797}" name="Description_GPT" dataDxfId="31"/>
-    <tableColumn id="5" xr3:uid="{1806E074-6CB5-47AB-8FA3-EF0F6E429062}" name="Underlying" dataDxfId="30"/>
-    <tableColumn id="7" xr3:uid="{21539C17-C1CC-4FA9-A0E1-A2F8FF8AB52C}" name="Active" dataDxfId="29"/>
-    <tableColumn id="37" xr3:uid="{DE50B7AE-5F67-471C-BE48-8BFA5076EDB0}" name="hyper_factor" dataDxfId="28"/>
-    <tableColumn id="10" xr3:uid="{494805E4-EBB6-47FD-9BC2-8DAD9FB9D3FA}" name="composite" dataDxfId="27"/>
-    <tableColumn id="14" xr3:uid="{608FE572-4016-436E-8625-08926F3A2371}" name="client" dataDxfId="26"/>
-    <tableColumn id="13" xr3:uid="{64EF0381-B0C5-4226-B34E-0F9752A4A840}" name="ticker" dataDxfId="25">
+    <tableColumn id="8" xr3:uid="{02943B27-7FCB-4450-B8E0-CF0DB6CF5CCA}" name="factor_name_new" dataDxfId="31"/>
+    <tableColumn id="4" xr3:uid="{D181BF84-863F-4FD0-B518-14EA5B0FB18E}" name="description_override" dataDxfId="30"/>
+    <tableColumn id="6" xr3:uid="{1C40DF9B-2910-4DE6-A188-563938E39797}" name="Description_GPT" dataDxfId="29"/>
+    <tableColumn id="5" xr3:uid="{1806E074-6CB5-47AB-8FA3-EF0F6E429062}" name="Underlying" dataDxfId="28"/>
+    <tableColumn id="7" xr3:uid="{21539C17-C1CC-4FA9-A0E1-A2F8FF8AB52C}" name="Active" dataDxfId="27"/>
+    <tableColumn id="37" xr3:uid="{DE50B7AE-5F67-471C-BE48-8BFA5076EDB0}" name="hyper_factor" dataDxfId="26"/>
+    <tableColumn id="10" xr3:uid="{494805E4-EBB6-47FD-9BC2-8DAD9FB9D3FA}" name="composite" dataDxfId="25"/>
+    <tableColumn id="14" xr3:uid="{608FE572-4016-436E-8625-08926F3A2371}" name="client" dataDxfId="24"/>
+    <tableColumn id="13" xr3:uid="{64EF0381-B0C5-4226-B34E-0F9752A4A840}" name="ticker" dataDxfId="23">
       <calculatedColumnFormula>data[[#This Row],[factor_name]]</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="9" xr3:uid="{5A601067-D384-419C-A711-AD3034F77E28}" name="description" dataDxfId="24">
+    <tableColumn id="9" xr3:uid="{5A601067-D384-419C-A711-AD3034F77E28}" name="description" dataDxfId="22">
       <calculatedColumnFormula array="1">_xlfn.IFS(data[[#This Row],[description_override]]&lt;&gt;"",data[[#This Row],[description_override]],data[[#This Row],[Description_GPT]]&lt;&gt;"",data[[#This Row],[Description_GPT]],data[[#This Row],[Underlying]]&lt;&gt;"",data[[#This Row],[Underlying]],TRUE,"-")</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="18" xr3:uid="{073BDADC-3AC0-4FF9-9654-A316B2345A90}" name="short_name_yf" dataDxfId="23">
+    <tableColumn id="18" xr3:uid="{073BDADC-3AC0-4FF9-9654-A316B2345A90}" name="short_name_yf" dataDxfId="21">
       <calculatedColumnFormula>_xlfn.XLOOKUP(data[[#This Row],[ticker]],yf_desc[ticker],yf_desc[shortName],"-")</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="19" xr3:uid="{3A563104-B6B0-465C-9D22-154F5FEA1B83}" name="long_name_yf" dataDxfId="22">
+    <tableColumn id="19" xr3:uid="{3A563104-B6B0-465C-9D22-154F5FEA1B83}" name="long_name_yf" dataDxfId="20">
       <calculatedColumnFormula>_xlfn.XLOOKUP(data[[#This Row],[ticker]],yf_desc[ticker],yf_desc[longName],"-")</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="17" xr3:uid="{A3F200A1-E769-49BA-8121-88EAA1180E80}" name="summary_yf" dataDxfId="21">
+    <tableColumn id="17" xr3:uid="{A3F200A1-E769-49BA-8121-88EAA1180E80}" name="summary_yf" dataDxfId="19">
       <calculatedColumnFormula>_xlfn.XLOOKUP(data[[#This Row],[ticker]],yf_desc[ticker],yf_desc[longBusinessSummary],"-")</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="15" xr3:uid="{D49341AB-DA48-473E-8CCB-3A3D04AED743}" name="note" dataDxfId="20"/>
+    <tableColumn id="15" xr3:uid="{D49341AB-DA48-473E-8CCB-3A3D04AED743}" name="note" dataDxfId="18"/>
   </tableColumns>
   <tableStyleInfo name="Table Style 1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{F918301C-859F-40B7-9C3E-90E8F0495E68}" name="data_old" displayName="data_old" ref="A1:I45" totalsRowShown="0" headerRowDxfId="19" dataDxfId="18">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{F918301C-859F-40B7-9C3E-90E8F0495E68}" name="data_old" displayName="data_old" ref="A1:I45" totalsRowShown="0" headerRowDxfId="17" dataDxfId="16">
   <autoFilter ref="A1:I45" xr:uid="{6DAD1482-C63D-400D-9F51-F22A8E35CAD8}"/>
   <tableColumns count="9">
-    <tableColumn id="1" xr3:uid="{B19D2B17-9AC9-4F1B-B32E-D4F72AAE469F}" name="asset_class" dataDxfId="17"/>
-    <tableColumn id="2" xr3:uid="{2C7CF29D-8E72-4B0C-A212-31F2A25D75C9}" name="region" dataDxfId="16"/>
-    <tableColumn id="3" xr3:uid="{C7E89EEC-2B5D-4C94-9327-1AC8E33DE708}" name="factor_name" dataDxfId="15"/>
-    <tableColumn id="8" xr3:uid="{B3F9004A-8BEB-463E-A746-8189A2AC2B3E}" name="factor_name_new" dataDxfId="14"/>
-    <tableColumn id="4" xr3:uid="{51CD7FB3-58FE-4906-B73C-7726C0A9C471}" name="description_override" dataDxfId="13"/>
-    <tableColumn id="6" xr3:uid="{3CFF990B-3164-4533-821F-08CE7C6D82CA}" name="Description_GPT" dataDxfId="12"/>
-    <tableColumn id="5" xr3:uid="{DD86D53E-A9B4-4387-ABF9-F2625E77982D}" name="Underlying" dataDxfId="11"/>
-    <tableColumn id="7" xr3:uid="{D56FFF9A-72FF-42A4-B3D2-2F27AB16AF7A}" name="Active" dataDxfId="10"/>
-    <tableColumn id="9" xr3:uid="{8476DFDE-B4B1-4FD9-99B4-DF1F2ABBD7D5}" name="description" dataDxfId="9">
+    <tableColumn id="1" xr3:uid="{B19D2B17-9AC9-4F1B-B32E-D4F72AAE469F}" name="asset_class" dataDxfId="15"/>
+    <tableColumn id="2" xr3:uid="{2C7CF29D-8E72-4B0C-A212-31F2A25D75C9}" name="region" dataDxfId="14"/>
+    <tableColumn id="3" xr3:uid="{C7E89EEC-2B5D-4C94-9327-1AC8E33DE708}" name="factor_name" dataDxfId="13"/>
+    <tableColumn id="8" xr3:uid="{B3F9004A-8BEB-463E-A746-8189A2AC2B3E}" name="factor_name_new" dataDxfId="12"/>
+    <tableColumn id="4" xr3:uid="{51CD7FB3-58FE-4906-B73C-7726C0A9C471}" name="description_override" dataDxfId="11"/>
+    <tableColumn id="6" xr3:uid="{3CFF990B-3164-4533-821F-08CE7C6D82CA}" name="Description_GPT" dataDxfId="10"/>
+    <tableColumn id="5" xr3:uid="{DD86D53E-A9B4-4387-ABF9-F2625E77982D}" name="Underlying" dataDxfId="9"/>
+    <tableColumn id="7" xr3:uid="{D56FFF9A-72FF-42A4-B3D2-2F27AB16AF7A}" name="Active" dataDxfId="8"/>
+    <tableColumn id="9" xr3:uid="{8476DFDE-B4B1-4FD9-99B4-DF1F2ABBD7D5}" name="description" dataDxfId="7">
       <calculatedColumnFormula>IF(data_old[[#This Row],[description_override]]="",data_old[[#This Row],[Description_GPT]],data_old[[#This Row],[description_override]])</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -4617,169 +4612,169 @@
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="6" spans="1:20" x14ac:dyDescent="0.25">
-      <c r="A6" s="20" t="s">
+      <c r="A6" s="18" t="s">
         <v>322</v>
       </c>
-      <c r="B6" s="21" t="s">
+      <c r="B6" s="19" t="s">
         <v>316</v>
       </c>
-      <c r="C6" s="21" t="s">
+      <c r="C6" s="19" t="s">
         <v>2</v>
       </c>
-      <c r="D6" s="21" t="s">
+      <c r="D6" s="19" t="s">
         <v>466</v>
       </c>
-      <c r="E6" s="21" t="s">
+      <c r="E6" s="19" t="s">
         <v>464</v>
       </c>
-      <c r="F6" s="21" t="s">
+      <c r="F6" s="19" t="s">
         <v>468</v>
       </c>
-      <c r="G6" s="21" t="s">
+      <c r="G6" s="19" t="s">
         <v>325</v>
       </c>
-      <c r="H6" s="21" t="s">
+      <c r="H6" s="19" t="s">
         <v>323</v>
       </c>
-      <c r="I6" s="21" t="s">
+      <c r="I6" s="19" t="s">
         <v>148</v>
       </c>
-      <c r="J6" s="21" t="s">
+      <c r="J6" s="19" t="s">
         <v>101</v>
       </c>
-      <c r="K6" s="21" t="s">
+      <c r="K6" s="19" t="s">
         <v>151</v>
       </c>
-      <c r="L6" s="21" t="s">
+      <c r="L6" s="19" t="s">
         <v>428</v>
       </c>
-      <c r="M6" s="21" t="s">
+      <c r="M6" s="19" t="s">
         <v>445</v>
       </c>
-      <c r="N6" s="21" t="s">
+      <c r="N6" s="19" t="s">
         <v>486</v>
       </c>
-      <c r="O6" s="21" t="s">
+      <c r="O6" s="19" t="s">
         <v>465</v>
       </c>
-      <c r="P6" s="21" t="s">
+      <c r="P6" s="19" t="s">
         <v>19</v>
       </c>
-      <c r="Q6" s="21" t="s">
+      <c r="Q6" s="19" t="s">
         <v>661</v>
       </c>
-      <c r="R6" s="21" t="s">
+      <c r="R6" s="19" t="s">
         <v>660</v>
       </c>
-      <c r="S6" s="21" t="s">
+      <c r="S6" s="19" t="s">
         <v>662</v>
       </c>
-      <c r="T6" s="22" t="s">
+      <c r="T6" s="20" t="s">
         <v>490</v>
       </c>
     </row>
     <row r="7" spans="1:20" x14ac:dyDescent="0.25">
-      <c r="A7" s="17" t="s">
+      <c r="A7" s="16" t="s">
         <v>444</v>
       </c>
-      <c r="B7" s="18" t="s">
+      <c r="B7" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="C7" s="18" t="s">
+      <c r="C7" s="4" t="s">
         <v>507</v>
       </c>
-      <c r="D7" s="18" t="s">
+      <c r="D7" s="4" t="s">
         <v>445</v>
       </c>
-      <c r="E7" s="18" t="s">
+      <c r="E7" s="4" t="s">
         <v>454</v>
       </c>
-      <c r="F7" s="18" cm="1">
+      <c r="F7" s="4" cm="1">
         <f t="array" ref="F7">_xlfn.SWITCH(data[[#This Row],[diffusion_type]],"lognormal",0.0001,"normal",-0.01)*IF(data[[#This Row],[asset_class]]="Vol",1,1)</f>
         <v>1E-4</v>
       </c>
-      <c r="G7" s="18"/>
-      <c r="H7" s="18"/>
-      <c r="I7" s="18"/>
-      <c r="J7" s="18" t="e" cm="1">
+      <c r="G7" s="4"/>
+      <c r="H7" s="4"/>
+      <c r="I7" s="4"/>
+      <c r="J7" s="4" t="e" cm="1">
         <f t="array" ref="J7">_xlfn.XLOOKUP(data[[#This Row],[factor_name]],_xlfn.ANCHORARRAY(composites!$I$2),_xlfn.ANCHORARRAY(composites!$J$2))</f>
         <v>#N/A</v>
       </c>
-      <c r="K7" s="18">
-        <v>1</v>
-      </c>
-      <c r="L7" s="18">
-        <v>0</v>
-      </c>
-      <c r="M7" s="18">
-        <v>0</v>
-      </c>
-      <c r="N7" s="18">
-        <v>0</v>
-      </c>
-      <c r="O7" s="18" t="str">
+      <c r="K7" s="4">
+        <v>1</v>
+      </c>
+      <c r="L7" s="4">
+        <v>0</v>
+      </c>
+      <c r="M7" s="4">
+        <v>0</v>
+      </c>
+      <c r="N7" s="4">
+        <v>0</v>
+      </c>
+      <c r="O7" s="4" t="str">
         <f>data[[#This Row],[factor_name]]</f>
         <v>DIA</v>
       </c>
-      <c r="P7" s="18" t="str" cm="1">
+      <c r="P7" s="4" t="str" cm="1">
         <f t="array" ref="P7">_xlfn.IFS(data[[#This Row],[description_override]]&lt;&gt;"",data[[#This Row],[description_override]],data[[#This Row],[Description_GPT]]&lt;&gt;"",data[[#This Row],[Description_GPT]],data[[#This Row],[Underlying]]&lt;&gt;"",data[[#This Row],[Underlying]],TRUE,"-")</f>
         <v>Dow Jones 30</v>
       </c>
-      <c r="Q7" s="18" t="str">
+      <c r="Q7" s="4" t="str">
         <f>_xlfn.XLOOKUP(data[[#This Row],[ticker]],yf_desc[ticker],yf_desc[shortName],"-")</f>
         <v>SPDR Dow Jones Industrial Avera</v>
       </c>
-      <c r="R7" s="18" t="str">
+      <c r="R7" s="4" t="str">
         <f>_xlfn.XLOOKUP(data[[#This Row],[ticker]],yf_desc[ticker],yf_desc[longName],"-")</f>
         <v>SPDR Dow Jones Industrial Average ETF Trust</v>
       </c>
-      <c r="S7" s="18" t="str">
+      <c r="S7" s="4" t="str">
         <f>_xlfn.XLOOKUP(data[[#This Row],[ticker]],yf_desc[ticker],yf_desc[longBusinessSummary],"-")</f>
         <v>The Trust’s Portfolio consists of substantially all of the component common stocks that comprise the DJIA, which are weighted in accordance with the terms of the Trust Agreement.</v>
       </c>
-      <c r="T7" s="19"/>
+      <c r="T7" s="17"/>
     </row>
     <row r="12" spans="1:20" x14ac:dyDescent="0.25">
-      <c r="A12" s="14" t="s">
+      <c r="A12" s="13" t="s">
         <v>507</v>
       </c>
       <c r="B12" s="1" t="s">
         <v>175</v>
       </c>
-      <c r="C12" s="15">
+      <c r="C12" s="14">
         <v>1.5</v>
       </c>
     </row>
     <row r="13" spans="1:20" x14ac:dyDescent="0.25">
-      <c r="A13" s="13" t="s">
+      <c r="A13" s="12" t="s">
         <v>507</v>
       </c>
-      <c r="B13" s="12" t="s">
+      <c r="B13" t="s">
         <v>431</v>
       </c>
-      <c r="C13" s="16">
+      <c r="C13" s="15">
         <v>-1</v>
       </c>
     </row>
     <row r="14" spans="1:20" x14ac:dyDescent="0.25">
-      <c r="A14" s="13" t="s">
+      <c r="A14" s="12" t="s">
         <v>507</v>
       </c>
-      <c r="B14" s="12" t="s">
+      <c r="B14" t="s">
         <v>5</v>
       </c>
-      <c r="C14" s="16">
+      <c r="C14" s="15">
         <v>1.5</v>
       </c>
     </row>
     <row r="15" spans="1:20" x14ac:dyDescent="0.25">
-      <c r="A15" s="13" t="s">
+      <c r="A15" s="12" t="s">
         <v>507</v>
       </c>
-      <c r="B15" s="12" t="s">
+      <c r="B15" t="s">
         <v>13</v>
       </c>
-      <c r="C15" s="16">
+      <c r="C15" s="15">
         <v>-1</v>
       </c>
     </row>
@@ -4802,9 +4797,7 @@
     <col min="1" max="1" width="15.42578125" customWidth="1"/>
     <col min="2" max="2" width="13.28515625" customWidth="1"/>
     <col min="3" max="3" width="12" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="12" customWidth="1"/>
-    <col min="5" max="6" width="12" style="23" customWidth="1"/>
-    <col min="7" max="13" width="12" customWidth="1"/>
+    <col min="4" max="13" width="12" customWidth="1"/>
     <col min="22" max="22" width="29.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -4835,7 +4828,7 @@
       <c r="C2">
         <v>1</v>
       </c>
-      <c r="E2" s="23" cm="1">
+      <c r="E2" cm="1">
         <f t="array" ref="E2:E28">_xlfn.XLOOKUP(composities[portfolio_name],data[factor_name],data[Active])</f>
         <v>1</v>
       </c>
@@ -4878,7 +4871,7 @@
       <c r="C3">
         <v>1</v>
       </c>
-      <c r="E3" s="23">
+      <c r="E3">
         <v>1</v>
       </c>
       <c r="H3" t="str">
@@ -4914,7 +4907,7 @@
       <c r="C4">
         <v>1</v>
       </c>
-      <c r="E4" s="23">
+      <c r="E4">
         <v>1</v>
       </c>
       <c r="H4" t="str">
@@ -4953,7 +4946,7 @@
       <c r="C5">
         <v>0.25</v>
       </c>
-      <c r="E5" s="23">
+      <c r="E5">
         <v>1</v>
       </c>
       <c r="H5" t="str">
@@ -4989,7 +4982,7 @@
       <c r="C6">
         <v>-0.25</v>
       </c>
-      <c r="E6" s="23">
+      <c r="E6">
         <v>1</v>
       </c>
       <c r="H6" t="str">
@@ -5025,7 +5018,7 @@
       <c r="C7">
         <v>0.65</v>
       </c>
-      <c r="E7" s="23">
+      <c r="E7">
         <v>1</v>
       </c>
       <c r="H7" t="str">
@@ -5064,7 +5057,7 @@
       <c r="C8">
         <v>0.3</v>
       </c>
-      <c r="E8" s="23">
+      <c r="E8">
         <v>1</v>
       </c>
       <c r="H8" t="str">
@@ -5106,7 +5099,7 @@
       <c r="C9">
         <v>-0.15</v>
       </c>
-      <c r="E9" s="23">
+      <c r="E9">
         <v>1</v>
       </c>
       <c r="H9" t="str">
@@ -5145,10 +5138,10 @@
       <c r="C10">
         <v>-0.05</v>
       </c>
-      <c r="E10" s="23">
-        <v>1</v>
-      </c>
-      <c r="F10" s="23" t="s">
+      <c r="E10">
+        <v>1</v>
+      </c>
+      <c r="F10" t="s">
         <v>728</v>
       </c>
       <c r="H10" t="str">
@@ -5191,7 +5184,7 @@
         <f>-C12*Y15/Y13</f>
         <v>-3.8633879781420766</v>
       </c>
-      <c r="E11" s="23">
+      <c r="E11">
         <v>1</v>
       </c>
       <c r="H11" t="str">
@@ -5218,7 +5211,7 @@
       <c r="C12">
         <v>1</v>
       </c>
-      <c r="E12" s="23">
+      <c r="E12">
         <v>1</v>
       </c>
       <c r="H12" t="str">
@@ -5245,7 +5238,7 @@
       <c r="C13" s="8">
         <v>1</v>
       </c>
-      <c r="E13" s="23">
+      <c r="E13">
         <v>1</v>
       </c>
       <c r="H13" t="str">
@@ -5272,7 +5265,7 @@
       <c r="C14" s="8">
         <v>-1</v>
       </c>
-      <c r="E14" s="23">
+      <c r="E14">
         <v>1</v>
       </c>
       <c r="H14" t="str">
@@ -5294,7 +5287,7 @@
         <f t="array" ref="C15">O18/N18*$P$18/SUM(ABS(($O$18:$O$22)))</f>
         <v>0.20547945205479451</v>
       </c>
-      <c r="E15" s="23">
+      <c r="E15">
         <v>1</v>
       </c>
       <c r="H15" t="str">
@@ -5327,7 +5320,7 @@
         <v>0.29702970297029702</v>
       </c>
       <c r="D16" s="8"/>
-      <c r="E16" s="23">
+      <c r="E16">
         <v>1</v>
       </c>
       <c r="G16" s="8"/>
@@ -5365,7 +5358,7 @@
         <v>0.36585365853658536</v>
       </c>
       <c r="D17" s="8"/>
-      <c r="E17" s="23">
+      <c r="E17">
         <v>1</v>
       </c>
       <c r="G17" s="8"/>
@@ -5397,7 +5390,7 @@
         <v>-3.7499999999999999E-2</v>
       </c>
       <c r="D18" s="8"/>
-      <c r="E18" s="23">
+      <c r="E18">
         <v>1</v>
       </c>
       <c r="G18" s="8"/>
@@ -5440,7 +5433,7 @@
         <v>0.15</v>
       </c>
       <c r="D19" s="8"/>
-      <c r="E19" s="23">
+      <c r="E19">
         <v>1</v>
       </c>
       <c r="G19" s="8"/>
@@ -5479,7 +5472,7 @@
         <v>-0.15</v>
       </c>
       <c r="D20" s="8"/>
-      <c r="E20" s="23">
+      <c r="E20">
         <v>1</v>
       </c>
       <c r="G20" s="8"/>
@@ -5519,7 +5512,7 @@
         <v>1</v>
       </c>
       <c r="D21" s="8"/>
-      <c r="E21" s="23">
+      <c r="E21">
         <v>1</v>
       </c>
       <c r="G21" s="8"/>
@@ -5556,7 +5549,7 @@
         <v>1</v>
       </c>
       <c r="D22" s="8"/>
-      <c r="E22" s="23">
+      <c r="E22">
         <v>1</v>
       </c>
       <c r="G22" s="8"/>
@@ -5590,7 +5583,7 @@
         <v>-1</v>
       </c>
       <c r="D23" s="8"/>
-      <c r="E23" s="23">
+      <c r="E23">
         <v>1</v>
       </c>
       <c r="G23" s="8"/>
@@ -5617,7 +5610,7 @@
       <c r="C24" s="8">
         <v>1</v>
       </c>
-      <c r="E24" s="23">
+      <c r="E24">
         <v>1</v>
       </c>
       <c r="H24" t="str">
@@ -5638,7 +5631,7 @@
       <c r="C25" s="8">
         <v>0.5</v>
       </c>
-      <c r="E25" s="23">
+      <c r="E25">
         <v>1</v>
       </c>
       <c r="H25" t="str">
@@ -5659,7 +5652,7 @@
       <c r="C26" s="8">
         <v>-0.5</v>
       </c>
-      <c r="E26" s="23">
+      <c r="E26">
         <v>1</v>
       </c>
       <c r="H26" t="str">
@@ -5680,7 +5673,7 @@
       <c r="C27" s="8">
         <v>0.5</v>
       </c>
-      <c r="E27" s="23">
+      <c r="E27">
         <v>1</v>
       </c>
       <c r="H27" t="str">
@@ -5701,7 +5694,7 @@
       <c r="C28" s="8">
         <v>-0.5</v>
       </c>
-      <c r="E28" s="23">
+      <c r="E28">
         <v>1</v>
       </c>
       <c r="H28" t="str">
@@ -5895,14 +5888,14 @@
       <formula>$T15</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A32:C33">
-    <cfRule type="expression" dxfId="2" priority="42">
-      <formula>$T19</formula>
+  <conditionalFormatting sqref="A29:C31">
+    <cfRule type="expression" dxfId="2" priority="44">
+      <formula>$T21</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A29:C31">
-    <cfRule type="expression" dxfId="1" priority="44">
-      <formula>$T21</formula>
+  <conditionalFormatting sqref="A32:C33">
+    <cfRule type="expression" dxfId="1" priority="42">
+      <formula>$T19</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -5916,7 +5909,7 @@
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3C29859C-7358-4E2F-B5CC-7696F1DAC449}">
   <sheetPr codeName="Sheet7"/>
-  <dimension ref="A1:Y113"/>
+  <dimension ref="A1:Y107"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12.28515625" customWidth="1"/>
@@ -5931,64 +5924,64 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A1" s="20" t="s">
+      <c r="A1" s="18" t="s">
         <v>322</v>
       </c>
-      <c r="B1" s="21" t="s">
+      <c r="B1" s="19" t="s">
         <v>316</v>
       </c>
-      <c r="C1" s="21" t="s">
+      <c r="C1" s="19" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="21" t="s">
+      <c r="D1" s="19" t="s">
         <v>466</v>
       </c>
-      <c r="E1" s="21" t="s">
+      <c r="E1" s="19" t="s">
         <v>464</v>
       </c>
-      <c r="F1" s="21" t="s">
+      <c r="F1" s="19" t="s">
         <v>468</v>
       </c>
-      <c r="G1" s="21" t="s">
+      <c r="G1" s="19" t="s">
         <v>325</v>
       </c>
-      <c r="H1" s="21" t="s">
+      <c r="H1" s="19" t="s">
         <v>323</v>
       </c>
-      <c r="I1" s="21" t="s">
+      <c r="I1" s="19" t="s">
         <v>148</v>
       </c>
-      <c r="J1" s="21" t="s">
+      <c r="J1" s="19" t="s">
         <v>101</v>
       </c>
-      <c r="K1" s="21" t="s">
+      <c r="K1" s="19" t="s">
         <v>151</v>
       </c>
-      <c r="L1" s="21" t="s">
+      <c r="L1" s="19" t="s">
         <v>428</v>
       </c>
-      <c r="M1" s="21" t="s">
+      <c r="M1" s="19" t="s">
         <v>445</v>
       </c>
-      <c r="N1" s="21" t="s">
+      <c r="N1" s="19" t="s">
         <v>486</v>
       </c>
-      <c r="O1" s="21" t="s">
+      <c r="O1" s="19" t="s">
         <v>465</v>
       </c>
-      <c r="P1" s="21" t="s">
+      <c r="P1" s="19" t="s">
         <v>19</v>
       </c>
-      <c r="Q1" s="21" t="s">
+      <c r="Q1" s="19" t="s">
         <v>661</v>
       </c>
-      <c r="R1" s="21" t="s">
+      <c r="R1" s="19" t="s">
         <v>660</v>
       </c>
-      <c r="S1" s="21" t="s">
+      <c r="S1" s="19" t="s">
         <v>662</v>
       </c>
-      <c r="T1" s="22" t="s">
+      <c r="T1" s="20" t="s">
         <v>490</v>
       </c>
     </row>
@@ -12412,7 +12405,7 @@
         <v>530</v>
       </c>
       <c r="K105" s="4">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L105" s="4">
         <v>0</v>
@@ -12557,18 +12550,6 @@
         <v>-</v>
       </c>
       <c r="T107" s="4"/>
-    </row>
-    <row r="110" spans="1:20" x14ac:dyDescent="0.25">
-      <c r="E110" s="12"/>
-    </row>
-    <row r="111" spans="1:20" x14ac:dyDescent="0.25">
-      <c r="E111" s="12"/>
-    </row>
-    <row r="112" spans="1:20" x14ac:dyDescent="0.25">
-      <c r="E112" s="12"/>
-    </row>
-    <row r="113" spans="5:5" x14ac:dyDescent="0.25">
-      <c r="E113" s="12"/>
     </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>
@@ -12753,7 +12734,7 @@
 
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E5A64DEF-E706-4B9C-B282-71F34F86B3DF}">
-  <dimension ref="A1:J86"/>
+  <dimension ref="A1:J85"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="6" max="6" width="44.28515625" bestFit="1" customWidth="1"/>
@@ -12793,11 +12774,11 @@
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2" t="str" cm="1">
-        <f t="array" ref="A2:A86">_xlfn._xlws.FILTER(data[factor_name],data[Active])</f>
+        <f t="array" ref="A2:A85">_xlfn._xlws.FILTER(data[factor_name],data[Active])</f>
         <v>SPY</v>
       </c>
       <c r="B2" t="str" cm="1">
-        <f t="array" ref="B2:J86">INDEX(data[],_xlfn.XMATCH(_xlfn.ANCHORARRAY(A2),data[factor_name]),_xlfn.XMATCH(B1:J1,data[#Headers]))</f>
+        <f t="array" ref="B2:J85">INDEX(data[],_xlfn.XMATCH(_xlfn.ANCHORARRAY(A2),data[factor_name]),_xlfn.XMATCH(B1:J1,data[#Headers]))</f>
         <v>Equities</v>
       </c>
       <c r="C2" t="str">
@@ -15419,10 +15400,10 @@
     </row>
     <row r="84" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A84" t="str">
-        <v>UNCERTAINTY</v>
+        <v>BTC</v>
       </c>
       <c r="B84" t="str">
-        <v>Econ</v>
+        <v>Currencies</v>
       </c>
       <c r="C84" t="str">
         <v>USD</v>
@@ -15434,27 +15415,27 @@
         <v>0</v>
       </c>
       <c r="F84" t="str">
-        <v>Economic Policy Uncertainty Index for United States</v>
+        <v>-</v>
       </c>
       <c r="G84" t="str">
-        <v>fred</v>
+        <v>lmxl</v>
       </c>
       <c r="H84" t="str">
-        <v>USEPUINDXD</v>
+        <v>BTC1_price</v>
       </c>
       <c r="I84" t="str">
-        <v>normal</v>
+        <v>lognormal</v>
       </c>
       <c r="J84">
-        <v>0.01</v>
+        <v>1E-4</v>
       </c>
     </row>
     <row r="85" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A85" t="str">
-        <v>BTC</v>
+        <v>BTC_vol</v>
       </c>
       <c r="B85" t="str">
-        <v>Currencies</v>
+        <v>Vol</v>
       </c>
       <c r="C85" t="str">
         <v>USD</v>
@@ -15472,44 +15453,12 @@
         <v>lmxl</v>
       </c>
       <c r="H85" t="str">
-        <v>BTC1_price</v>
+        <v>BTC1_atm</v>
       </c>
       <c r="I85" t="str">
-        <v>lognormal</v>
+        <v>normal</v>
       </c>
       <c r="J85">
-        <v>1E-4</v>
-      </c>
-    </row>
-    <row r="86" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A86" t="str">
-        <v>BTC_vol</v>
-      </c>
-      <c r="B86" t="str">
-        <v>Vol</v>
-      </c>
-      <c r="C86" t="str">
-        <v>USD</v>
-      </c>
-      <c r="D86">
-        <v>0</v>
-      </c>
-      <c r="E86">
-        <v>0</v>
-      </c>
-      <c r="F86" t="str">
-        <v>-</v>
-      </c>
-      <c r="G86" t="str">
-        <v>lmxl</v>
-      </c>
-      <c r="H86" t="str">
-        <v>BTC1_atm</v>
-      </c>
-      <c r="I86" t="str">
-        <v>normal</v>
-      </c>
-      <c r="J86">
         <v>-0.01</v>
       </c>
     </row>
@@ -17904,7 +17853,7 @@
 <file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2977BD7F-9323-4F6D-98BF-C1B39119DCDE}">
   <sheetPr codeName="Sheet8"/>
-  <dimension ref="A1:J86"/>
+  <dimension ref="A1:J85"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="6" max="6" width="44.28515625" bestFit="1" customWidth="1"/>
@@ -17944,11 +17893,11 @@
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2" t="str" cm="1">
-        <f t="array" ref="A2:A86">_xlfn._xlws.FILTER(data[factor_name],data[Active]*(data[client]=0))</f>
+        <f t="array" ref="A2:A85">_xlfn._xlws.FILTER(data[factor_name],data[Active]*(data[client]=0))</f>
         <v>SPY</v>
       </c>
       <c r="B2" t="str" cm="1">
-        <f t="array" ref="B2:J86">INDEX(data[],_xlfn.XMATCH(_xlfn.ANCHORARRAY(A2),data[factor_name]),_xlfn.XMATCH(B1:J1,data[#Headers]))</f>
+        <f t="array" ref="B2:J85">INDEX(data[],_xlfn.XMATCH(_xlfn.ANCHORARRAY(A2),data[factor_name]),_xlfn.XMATCH(B1:J1,data[#Headers]))</f>
         <v>Equities</v>
       </c>
       <c r="C2" t="str">
@@ -20570,10 +20519,10 @@
     </row>
     <row r="84" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A84" t="str">
-        <v>UNCERTAINTY</v>
+        <v>BTC</v>
       </c>
       <c r="B84" t="str">
-        <v>Econ</v>
+        <v>Currencies</v>
       </c>
       <c r="C84" t="str">
         <v>USD</v>
@@ -20585,27 +20534,27 @@
         <v>0</v>
       </c>
       <c r="F84" t="str">
-        <v>Economic Policy Uncertainty Index for United States</v>
+        <v>-</v>
       </c>
       <c r="G84" t="str">
-        <v>fred</v>
+        <v>lmxl</v>
       </c>
       <c r="H84" t="str">
-        <v>USEPUINDXD</v>
+        <v>BTC1_price</v>
       </c>
       <c r="I84" t="str">
-        <v>normal</v>
+        <v>lognormal</v>
       </c>
       <c r="J84">
-        <v>0.01</v>
+        <v>1E-4</v>
       </c>
     </row>
     <row r="85" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A85" t="str">
-        <v>BTC</v>
+        <v>BTC_vol</v>
       </c>
       <c r="B85" t="str">
-        <v>Currencies</v>
+        <v>Vol</v>
       </c>
       <c r="C85" t="str">
         <v>USD</v>
@@ -20623,44 +20572,12 @@
         <v>lmxl</v>
       </c>
       <c r="H85" t="str">
-        <v>BTC1_price</v>
+        <v>BTC1_atm</v>
       </c>
       <c r="I85" t="str">
-        <v>lognormal</v>
+        <v>normal</v>
       </c>
       <c r="J85">
-        <v>1E-4</v>
-      </c>
-    </row>
-    <row r="86" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A86" t="str">
-        <v>BTC_vol</v>
-      </c>
-      <c r="B86" t="str">
-        <v>Vol</v>
-      </c>
-      <c r="C86" t="str">
-        <v>USD</v>
-      </c>
-      <c r="D86">
-        <v>0</v>
-      </c>
-      <c r="E86">
-        <v>0</v>
-      </c>
-      <c r="F86" t="str">
-        <v>-</v>
-      </c>
-      <c r="G86" t="str">
-        <v>lmxl</v>
-      </c>
-      <c r="H86" t="str">
-        <v>BTC1_atm</v>
-      </c>
-      <c r="I86" t="str">
-        <v>normal</v>
-      </c>
-      <c r="J86">
         <v>-0.01</v>
       </c>
     </row>
@@ -20878,7 +20795,7 @@
 <file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D1A08F2F-299B-47F7-8064-36693758F4E3}">
   <sheetPr codeName="Sheet9"/>
-  <dimension ref="A1:E77"/>
+  <dimension ref="A1:E76"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="5" max="5" width="44.28515625" bestFit="1" customWidth="1"/>
@@ -20903,11 +20820,11 @@
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" t="str" cm="1">
-        <f t="array" ref="A2:A77">_xlfn._xlws.FILTER(data[factor_name],data[Active]*NOT(data[composite]))</f>
+        <f t="array" ref="A2:A76">_xlfn._xlws.FILTER(data[factor_name],data[Active]*NOT(data[composite]))</f>
         <v>SPY</v>
       </c>
       <c r="B2" t="str" cm="1">
-        <f t="array" ref="B2:E77">INDEX(data[],_xlfn.XMATCH(_xlfn.ANCHORARRAY(A2),data[factor_name]),_xlfn.XMATCH(B1:E1,data[#Headers]))</f>
+        <f t="array" ref="B2:E76">INDEX(data[],_xlfn.XMATCH(_xlfn.ANCHORARRAY(A2),data[factor_name]),_xlfn.XMATCH(B1:E1,data[#Headers]))</f>
         <v>Equities</v>
       </c>
       <c r="C2" t="str">
@@ -22146,10 +22063,10 @@
     </row>
     <row r="75" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A75" t="str">
-        <v>UNCERTAINTY</v>
+        <v>BTC</v>
       </c>
       <c r="B75" t="str">
-        <v>Econ</v>
+        <v>Currencies</v>
       </c>
       <c r="C75" t="str">
         <v>USD</v>
@@ -22158,15 +22075,15 @@
         <v>0</v>
       </c>
       <c r="E75" t="str">
-        <v>Economic Policy Uncertainty Index for United States</v>
+        <v>-</v>
       </c>
     </row>
     <row r="76" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A76" t="str">
-        <v>BTC</v>
+        <v>BTC_vol</v>
       </c>
       <c r="B76" t="str">
-        <v>Currencies</v>
+        <v>Vol</v>
       </c>
       <c r="C76" t="str">
         <v>USD</v>
@@ -22175,23 +22092,6 @@
         <v>0</v>
       </c>
       <c r="E76" t="str">
-        <v>-</v>
-      </c>
-    </row>
-    <row r="77" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A77" t="str">
-        <v>BTC_vol</v>
-      </c>
-      <c r="B77" t="str">
-        <v>Vol</v>
-      </c>
-      <c r="C77" t="str">
-        <v>USD</v>
-      </c>
-      <c r="D77">
-        <v>0</v>
-      </c>
-      <c r="E77" t="str">
         <v>-</v>
       </c>
     </row>
@@ -27903,7 +27803,7 @@
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="10">
         <f ca="1">TODAY()-1</f>
-        <v>46131</v>
+        <v>46186</v>
       </c>
       <c r="B2">
         <v>0.20547945205479451</v>

</xml_diff>